<commit_message>
auto-publish commission xlsx: manual
</commit_message>
<xml_diff>
--- a/commission/karin/2026-07.xlsx
+++ b/commission/karin/2026-07.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="58">
   <si>
     <t>Equine Performance Labs, LLC</t>
   </si>
@@ -37,6 +37,12 @@
     <t>Q3 Route C Accelerator — tiered on invoiced revenue when $30K gate met (else standard waterfall)</t>
   </si>
   <si>
+    <t>Basis</t>
+  </si>
+  <si>
+    <t>✅ CRM + QuickBooks reconciled (paid on cleared)</t>
+  </si>
+  <si>
     <t>Route C — Q3 Accelerator</t>
   </si>
   <si>
@@ -140,6 +146,42 @@
   </si>
   <si>
     <t>ORD-EPL-1143</t>
+  </si>
+  <si>
+    <t>ADJUSTMENTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Austin Equine Clinic</t>
+  </si>
+  <si>
+    <t>QB deposit cleared 7/7/2026 on June-dated invoice (CINV-EPL-1018 dated 6/8/2026); missing from CRM Received Payments July export. Rate: 5% (Route C fallback — gate missed, standard waterfall tier 1).</t>
+  </si>
+  <si>
+    <t>CINV-EPL-1018</t>
+  </si>
+  <si>
+    <t>QB deposit cleared 7/7/2026 on June-dated invoice (CINV-EPL-1019 dated 6/8/2026); missing from CRM Received Payments July export. Rate: 5% (Route C fallback — gate missed, standard waterfall tier 1).</t>
+  </si>
+  <si>
+    <t>CINV-EPL-1019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Elgin Equine</t>
+  </si>
+  <si>
+    <t>QB deposit cleared 7/24/2026 on 7/1/2026 invoice (ORD-EPL-1129); missing from CRM Received Payments July export. Rate: 5% (Route C fallback — gate missed, standard waterfall tier 1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Signature S Equine</t>
+  </si>
+  <si>
+    <t>QB deposit cleared 7/27/2026 — prepayment on 8/7/2026 invoice (ORD-EPL-1171). Missing from CRM Received Payments July export. Rate: 5% (Route C fallback — gate missed, standard waterfall tier 1). Commissionable in July (payment received basis).</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1171</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Adjustments subtotal</t>
   </si>
   <si>
     <t>GRAND TOTAL</t>
@@ -149,12 +191,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -186,6 +229,11 @@
     <font>
       <b/>
       <color rgb="0F5E4F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="0F5E4F"/>
       <sz val="12"/>
     </font>
     <font>
@@ -212,12 +260,22 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="7A7974"/>
+    </font>
+    <font>
       <b/>
-      <color rgb="0F5E4F"/>
+      <color rgb="7A5C1C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="7A5C1C"/>
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="7A7974"/>
+      <b/>
+      <i/>
+      <sz val="10"/>
     </font>
     <font>
       <b/>
@@ -254,7 +312,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -262,21 +320,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -287,7 +346,19 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -632,7 +703,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -653,7 +724,7 @@
         <v>1</v>
       </c>
       <c r="H1" s="3">
-        <v>753.75</v>
+        <v>933.75</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -678,404 +749,508 @@
         <v>7</v>
       </c>
     </row>
+    <row r="4" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>8</v>
+      <c r="A5" s="7" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="7">
+        <v>11</v>
+      </c>
+      <c r="B6" s="8">
         <v>15075</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>10</v>
+      <c r="C6" s="9" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="10">
+      <c r="A7" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="11">
         <v>753.75</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="B9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="C9" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="D9" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="E9" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="F9" s="13" t="s">
         <v>19</v>
       </c>
+      <c r="G9" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="14">
+      <c r="A10" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="15">
         <v>4800</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="16">
         <v>720</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="16">
+      <c r="B11" s="17">
         <v>46226.5</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F11" s="17">
+        <v>24</v>
+      </c>
+      <c r="F11" s="18">
         <v>0</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="G11" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="17">
+        <v>46226.5</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="E12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="18">
+        <v>4800</v>
+      </c>
+      <c r="G12" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="15">
+        <v>3600</v>
+      </c>
+      <c r="H14" s="16">
+        <v>397.5</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="17">
+        <v>46224.5</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="16">
-        <v>46226.5</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="17">
-        <v>4800</v>
-      </c>
-      <c r="G12" s="18" t="s">
+      <c r="E15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="18">
+        <v>1800</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="17">
+        <v>46204.5</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="E16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="18">
+        <v>1800</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="15">
+        <v>1800</v>
+      </c>
+      <c r="H18" s="16">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="17">
+        <v>46218.5</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="14">
+      <c r="E19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" s="18">
+        <v>1800</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H19" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="15">
+        <v>1800</v>
+      </c>
+      <c r="H21" s="16">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="17">
+        <v>46210.5</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F22" s="18">
+        <v>1800</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H22" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" s="15">
+        <v>1275</v>
+      </c>
+      <c r="H24" s="16">
+        <v>140.78</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="17">
+        <v>46210.5</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" s="18">
+        <v>1275</v>
+      </c>
+      <c r="G25" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="F27" s="15">
+        <v>1200</v>
+      </c>
+      <c r="H27" s="16">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="17">
+        <v>46225.5</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" s="18">
+        <v>1200</v>
+      </c>
+      <c r="G28" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H28" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F30" s="15">
+        <v>600</v>
+      </c>
+      <c r="H30" s="16">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" s="17">
+        <v>46211.5</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F31" s="18">
+        <v>600</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H31" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F33" s="15">
+        <v>0</v>
+      </c>
+      <c r="H33" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B34" s="17">
+        <v>46225.5</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F34" s="18">
+        <v>0</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B35" s="17">
+        <v>46209.5</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F35" s="18">
+        <v>0</v>
+      </c>
+      <c r="G35" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H35" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F37" s="15">
+        <v>0</v>
+      </c>
+      <c r="H37" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B38" s="17">
+        <v>46223.5</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F38" s="18">
+        <v>0</v>
+      </c>
+      <c r="G38" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H38" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D43" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F43" s="22">
+        <v>600</v>
+      </c>
+      <c r="G43" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="H43" s="22">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D44" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F44" s="22">
+        <v>600</v>
+      </c>
+      <c r="G44" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="H44" s="22">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D45" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F45" s="22">
+        <v>1800</v>
+      </c>
+      <c r="G45" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="H45" s="22">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D46" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F46" s="22">
+        <v>600</v>
+      </c>
+      <c r="G46" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="H46" s="22">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="F47" s="25">
         <v>3600</v>
       </c>
-      <c r="H14" s="15">
-        <v>397.5</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="16">
-        <v>46224.5</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F15" s="17">
-        <v>1800</v>
-      </c>
-      <c r="G15" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="16">
-        <v>46204.5</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="17">
-        <v>1800</v>
-      </c>
-      <c r="G16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="F18" s="14">
-        <v>1800</v>
-      </c>
-      <c r="H18" s="15">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="16">
-        <v>46218.5</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F19" s="17">
-        <v>1800</v>
-      </c>
-      <c r="G19" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F21" s="14">
-        <v>1800</v>
-      </c>
-      <c r="H21" s="15">
+      <c r="H47" s="25">
         <v>180</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="16">
-        <v>46210.5</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F22" s="17">
-        <v>1800</v>
-      </c>
-      <c r="G22" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H22" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F24" s="14">
-        <v>1275</v>
-      </c>
-      <c r="H24" s="15">
-        <v>140.78</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="16">
-        <v>46210.5</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F25" s="17">
-        <v>1275</v>
-      </c>
-      <c r="G25" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H25" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F27" s="14">
-        <v>1200</v>
-      </c>
-      <c r="H27" s="15">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="16">
-        <v>46225.5</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F28" s="17">
-        <v>1200</v>
-      </c>
-      <c r="G28" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H28" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="F30" s="14">
-        <v>600</v>
-      </c>
-      <c r="H30" s="15">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B31" s="16">
-        <v>46211.5</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F31" s="17">
-        <v>600</v>
-      </c>
-      <c r="G31" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H31" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="F33" s="14">
-        <v>0</v>
-      </c>
-      <c r="H33" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="16">
-        <v>46225.5</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F34" s="17">
-        <v>0</v>
-      </c>
-      <c r="G34" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H34" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="16">
-        <v>46209.5</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F35" s="17">
-        <v>0</v>
-      </c>
-      <c r="G35" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H35" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="F37" s="14">
-        <v>0</v>
-      </c>
-      <c r="H37" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B38" s="16">
-        <v>46223.5</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F38" s="17">
-        <v>0</v>
-      </c>
-      <c r="G38" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H38" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="F41" s="20">
-        <v>15075</v>
-      </c>
-      <c r="H41" s="21">
-        <v>753.75</v>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="F48" s="27">
+        <v>18675</v>
+      </c>
+      <c r="H48" s="28">
+        <v>933.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>